<commit_message>
Add API endpoints for viewing and exporting accepted students list in Sprint 3.
Implemented the GET endpoints to retrieve and export accepted applications as CSV, fully verified by unit tests for accurate data filtering and 403 unauthorized access prevention.
</commit_message>
<xml_diff>
--- a/test-evidence/M6-Yin-Mingze/UT-M6-table.xlsx
+++ b/test-evidence/M6-Yin-Mingze/UT-M6-table.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="33">
   <si>
     <t>Test Name/ID</t>
   </si>
@@ -98,31 +98,34 @@
     <t>Sprint 3</t>
   </si>
   <si>
-    <t>Application ID does not exist in the database.</t>
-  </si>
-  <si>
-    <t>processApproval(99L, true)</t>
-  </si>
-  <si>
-    <t>Throws Exception.</t>
-  </si>
-  <si>
-    <t>System throws a RuntimeException with message "Application not found".</t>
-  </si>
-  <si>
-    <t>RuntimeException thrown with message "Application not found".</t>
+    <t>Topic ID 100 belongs to Teacher ID 10. Student applications exist with accepted status.</t>
+  </si>
+  <si>
+    <t>HTTP GET request to /api/teacher/applications/topics/100/students?teacherId=10</t>
+  </si>
+  <si>
+    <t>JSON list containing only applications with accepted status.</t>
+  </si>
+  <si>
+    <t>HTTP Status Code: 200 OK.</t>
+  </si>
+  <si>
+    <t>Returned HTTP 200 OK and the correctly filtered list of accepted students.</t>
   </si>
   <si>
     <t>UT-M6-S3-02</t>
   </si>
   <si>
-    <t>Application (ID=1) exists but its status is NOT pending (e.g., already accepted).</t>
-  </si>
-  <si>
-    <t>System throws a RuntimeException with message "Only pending applications can be processed".</t>
-  </si>
-  <si>
-    <t>RuntimeException thrown with message "Only pending applications can be processed".</t>
+    <t>HTTP GET request to /api/teacher/applications/topics/100/students?teacherId=99 (Unauthorized teacher ID)</t>
+  </si>
+  <si>
+    <t>System intercepts the request and throws an unauthorized exception.</t>
+  </si>
+  <si>
+    <t>HTTP Status Code: 403 Forbidden.</t>
+  </si>
+  <si>
+    <t>Successfully intercepted unauthorized access and returned HTTP 403.</t>
   </si>
 </sst>
 </file>
@@ -135,7 +138,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -147,13 +150,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -303,7 +299,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -331,12 +327,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -633,67 +623,70 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -708,73 +701,70 @@
     <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1256,19 +1246,19 @@
         <v>22</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>15</v>

</xml_diff>